<commit_message>
Tobacco Research bug fix and ADAE field changes
</commit_message>
<xml_diff>
--- a/static/fields/animalandveterinaryevent_reference.xlsx
+++ b/static/fields/animalandveterinaryevent_reference.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10709"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="11214"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jackfinch/WebstormProjects/open.fda.gov/static/fields/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/violet.wren/WebstormProjects/open.fda.gov/static/fields/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65F5D0CA-6345-604C-BBDB-42396DD6E657}" xr6:coauthVersionLast="34" xr6:coauthVersionMax="34" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{780FC8C0-BEC1-8F4B-8ADE-995902397B6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="560" yWindow="460" windowWidth="28240" windowHeight="15820" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="560" yWindow="500" windowWidth="28240" windowHeight="15820" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="drug_event_fields" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="166">
   <si>
     <t>Field Name</t>
   </si>
@@ -517,6 +517,12 @@
   </si>
   <si>
     <t>Note: MSK is a null flavor that means "masked." MSK is used when there is information available for the value, but it has not been provided to the sender due to security, privacy, or other reasons.</t>
+  </si>
+  <si>
+    <t>foreign_or_domestic</t>
+  </si>
+  <si>
+    <t>A flag indicating whether the product is foreign or domestic.</t>
   </si>
 </sst>
 </file>
@@ -682,28 +688,28 @@
   </cellStyleXfs>
   <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -1146,7 +1152,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D82"/>
+  <dimension ref="A1:D83"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="33.5" style="3" bestFit="1" customWidth="1"/>
@@ -1673,7 +1679,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="39" spans="1:4" ht="32" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:4" ht="51" x14ac:dyDescent="0.2">
       <c r="A39" s="3" t="s">
         <v>80</v>
       </c>
@@ -1687,7 +1693,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A40" s="3" t="s">
         <v>46</v>
       </c>
@@ -1701,7 +1707,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A41" s="3" t="s">
         <v>46</v>
       </c>
@@ -1715,7 +1721,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A42" s="3" t="s">
         <v>46</v>
       </c>
@@ -1729,7 +1735,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A43" s="3" t="s">
         <v>46</v>
       </c>
@@ -1743,7 +1749,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="44" spans="1:4" ht="32" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:4" ht="51" x14ac:dyDescent="0.2">
       <c r="A44" s="3" t="s">
         <v>46</v>
       </c>
@@ -1757,7 +1763,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="45" spans="1:4" ht="32" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:4" ht="51" x14ac:dyDescent="0.2">
       <c r="A45" s="3" t="s">
         <v>46</v>
       </c>
@@ -1771,7 +1777,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A46" s="3" t="s">
         <v>46</v>
       </c>
@@ -1785,7 +1791,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A47" s="3" t="s">
         <v>46</v>
       </c>
@@ -1799,7 +1805,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="48" spans="1:4" ht="32" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A48" s="3" t="s">
         <v>46</v>
       </c>
@@ -1813,7 +1819,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="B49" s="4" t="s">
         <v>101</v>
       </c>
@@ -1824,7 +1830,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A50" s="3" t="s">
         <v>101</v>
       </c>
@@ -1838,7 +1844,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A51" s="3" t="s">
         <v>101</v>
       </c>
@@ -1852,7 +1858,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="52" spans="1:4" ht="32" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:4" ht="51" x14ac:dyDescent="0.2">
       <c r="B52" s="4" t="s">
         <v>105</v>
       </c>
@@ -1863,7 +1869,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A53" s="3" t="s">
         <v>105</v>
       </c>
@@ -1877,7 +1883,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A54" s="3" t="s">
         <v>105</v>
       </c>
@@ -1891,7 +1897,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="55" spans="1:4" ht="32" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="B55" s="4" t="s">
         <v>111</v>
       </c>
@@ -1902,7 +1908,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="B56" s="4" t="s">
         <v>113</v>
       </c>
@@ -1913,7 +1919,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="B57" s="4" t="s">
         <v>115</v>
       </c>
@@ -1924,7 +1930,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="B58" s="4" t="s">
         <v>117</v>
       </c>
@@ -1935,306 +1941,317 @@
         <v>118</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="B59" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="C59" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D59" s="5" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="B60" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="C59" s="3" t="s">
+      <c r="C60" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D59" s="5" t="s">
+      <c r="D60" s="5" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A60" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="B60" s="4" t="s">
-        <v>121</v>
-      </c>
-      <c r="C60" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="D60" s="5" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="61" spans="1:4" ht="32" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A61" s="3" t="s">
         <v>119</v>
       </c>
       <c r="B61" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="C61" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D61" s="5" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="A62" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="B62" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="C61" s="3" t="s">
+      <c r="C62" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="D61" s="5" t="s">
+      <c r="D62" s="5" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B62" s="4" t="s">
+    <row r="63" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="B63" s="4" t="s">
         <v>123</v>
       </c>
-      <c r="C62" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="D62" s="5" t="s">
+      <c r="C63" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D63" s="5" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B63" s="4" t="s">
+    <row r="64" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="B64" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="C63" s="3" t="s">
+      <c r="C64" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D63" s="5" t="s">
+      <c r="D64" s="5" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A64" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="B64" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="C64" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="D64" s="5" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="65" spans="1:4" ht="32" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A65" s="3" t="s">
         <v>125</v>
       </c>
       <c r="B65" s="4" t="s">
-        <v>111</v>
+        <v>127</v>
       </c>
       <c r="C65" s="3" t="s">
-        <v>87</v>
+        <v>3</v>
       </c>
       <c r="D65" s="5" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.2">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A66" s="3" t="s">
         <v>125</v>
       </c>
       <c r="B66" s="4" t="s">
-        <v>129</v>
+        <v>111</v>
       </c>
       <c r="C66" s="3" t="s">
-        <v>3</v>
+        <v>87</v>
       </c>
       <c r="D66" s="5" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.2">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A67" s="3" t="s">
         <v>125</v>
       </c>
       <c r="B67" s="4" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="C67" s="3" t="s">
         <v>3</v>
       </c>
       <c r="D67" s="5" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.2">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A68" s="3" t="s">
         <v>125</v>
       </c>
       <c r="B68" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="C68" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D68" s="5" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="A69" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="B69" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="C68" s="3" t="s">
+      <c r="C69" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="D68" s="5" t="s">
+      <c r="D69" s="5" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B69" s="4" t="s">
+    <row r="70" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="B70" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="C69" s="3" t="s">
+      <c r="C70" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D69" s="5" t="s">
+      <c r="D70" s="5" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A70" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="B70" s="4" t="s">
-        <v>138</v>
-      </c>
-      <c r="C70" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="D70" s="5" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A71" s="3" t="s">
         <v>135</v>
       </c>
       <c r="B71" s="4" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C71" s="3" t="s">
         <v>3</v>
       </c>
       <c r="D71" s="5" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.2">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A72" s="3" t="s">
         <v>135</v>
       </c>
       <c r="B72" s="4" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C72" s="3" t="s">
         <v>3</v>
       </c>
       <c r="D72" s="5" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.2">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A73" s="3" t="s">
         <v>135</v>
       </c>
       <c r="B73" s="4" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="C73" s="3" t="s">
         <v>3</v>
       </c>
       <c r="D73" s="5" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.2">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A74" s="3" t="s">
         <v>135</v>
       </c>
       <c r="B74" s="4" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C74" s="3" t="s">
         <v>3</v>
       </c>
       <c r="D74" s="5" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.2">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A75" s="3" t="s">
         <v>135</v>
       </c>
       <c r="B75" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="C75" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D75" s="5" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A76" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="B76" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="C75" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="D75" s="5" t="s">
+      <c r="C76" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D76" s="5" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="76" spans="1:4" ht="48" x14ac:dyDescent="0.2">
-      <c r="B76" s="4" t="s">
+    <row r="77" spans="1:4" ht="85" x14ac:dyDescent="0.2">
+      <c r="B77" s="4" t="s">
         <v>149</v>
       </c>
-      <c r="C76" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="D76" s="5" t="s">
+      <c r="C77" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D77" s="5" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="77" spans="1:4" ht="32" x14ac:dyDescent="0.2">
-      <c r="B77" s="4" t="s">
+    <row r="78" spans="1:4" ht="51" x14ac:dyDescent="0.2">
+      <c r="B78" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="C77" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="D77" s="5" t="s">
+      <c r="C78" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D78" s="5" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B78" s="4" t="s">
+    <row r="79" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="B79" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="C78" s="3" t="s">
+      <c r="C79" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="D78" s="5" t="s">
+      <c r="D79" s="5" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B79" s="4" t="s">
+    <row r="80" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="B80" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="C79" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="D79" s="5" t="s">
+      <c r="C80" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D80" s="5" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B80" s="4" t="s">
+    <row r="81" spans="2:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="B81" s="4" t="s">
         <v>157</v>
       </c>
-      <c r="C80" s="3" t="s">
+      <c r="C81" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="D80" s="5" t="s">
+      <c r="D81" s="5" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="81" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B81" s="4" t="s">
+    <row r="82" spans="2:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="B82" s="4" t="s">
         <v>159</v>
       </c>
-      <c r="C81" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="D81" s="5" t="s">
+      <c r="C82" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D82" s="5" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="82" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B82" s="4" t="s">
+    <row r="83" spans="2:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="B83" s="4" t="s">
         <v>161</v>
       </c>
-      <c r="C82" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="D82" s="5" t="s">
+      <c r="C83" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D83" s="5" t="s">
         <v>162</v>
       </c>
     </row>

</xml_diff>